<commit_message>
Update Chapter 02: 未來教育與計劃
</commit_message>
<xml_diff>
--- a/content-pipeline/inputs/chapter02_final.xlsx
+++ b/content-pipeline/inputs/chapter02_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://transre-my.sharepoint.com/personal/fau_transre_com/Documents/_OneDrive/_Operational_Tools/Github/GCSEChinese/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{2A1A79E6-1D5A-44ED-B57F-878C872B756E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1E74013-568C-49EB-9065-032D7A8C1C7F}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="8_{2A1A79E6-1D5A-44ED-B57F-878C872B756E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83E01678-8AD8-4D62-97BB-B3A9ADB5AB9D}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1905" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -114,7 +114,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="122">
   <si>
     <t>Passage</t>
   </si>
@@ -476,6 +476,35 @@
   </si>
   <si>
     <t>這個朋友最後憑着自己的努力，終於過了一個充實的空檔年。</t>
+  </si>
+  <si>
+    <t>五湖四海</t>
+  </si>
+  <si>
+    <t>善用</t>
+  </si>
+  <si>
+    <t>all over the country</t>
+  </si>
+  <si>
+    <t>to make good use of</t>
+  </si>
+  <si>
+    <t>除了學習漢語以外，還可以認識到來自五湖四海的朋友，十分有意義。</t>
+  </si>
+  <si>
+    <t>如果你在中國的大學裏認識了一個在空檔年的國外學生，你會建議他如何善用這一年的時間？</t>
+  </si>
+  <si>
+    <t>很多國外的大學生都喜歡在空檔年到中國留學，除了學習漢語以外，還可以認識到來自五湖四海的朋友，十分有意義。
+1. 國外的大學生到中國留學一年，可以學到什麼？ 
+2. 如果你在中國的大學裏認識了一個在空檔年的國外學生，你會建議他如何善用這一年的時間？</t>
+  </si>
+  <si>
+    <t>wǔ hú sì hǎi</t>
+  </si>
+  <si>
+    <t>shàn yòng</t>
   </si>
 </sst>
 </file>
@@ -561,12 +590,12 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1008,8 +1037,10 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
+    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>119</v>
+      </c>
       <c r="B5" t="s">
         <v>10</v>
       </c>
@@ -1208,9 +1239,21 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
+      <c r="B27" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
+      <c r="B28" t="s">
+        <v>114</v>
+      </c>
+      <c r="C28" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
@@ -1277,14 +1320,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1294,20 +1337,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
@@ -1487,7 +1530,7 @@
       <c r="C15" t="s">
         <v>81</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="5" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1671,6 +1714,34 @@
       </c>
       <c r="D28" t="s">
         <v>112</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>113</v>
+      </c>
+      <c r="B29" t="s">
+        <v>115</v>
+      </c>
+      <c r="C29" t="s">
+        <v>120</v>
+      </c>
+      <c r="D29" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>114</v>
+      </c>
+      <c r="B30" t="s">
+        <v>116</v>
+      </c>
+      <c r="C30" t="s">
+        <v>121</v>
+      </c>
+      <c r="D30" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>